<commit_message>
V6 Release: Integrated payroll premiums, auto-calculation engine, yearly salary increase settings, and fixed shareholder report API routes
</commit_message>
<xml_diff>
--- a/Accounts 2026/Salaries Landco 2026/Landco Salaries 2026/02 Salary sheet for Landco.xlsx
+++ b/Accounts 2026/Salaries Landco 2026/Landco Salaries 2026/02 Salary sheet for Landco.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andrisa\Dropbox\Andrisa\Landco\Accounts 2026\Salaries Landco 2026\Landco Salaries 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\landco\Accounts 2026\Salaries Landco 2026\Landco Salaries 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B87B37-9567-4E31-9E0C-17016028BC56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F7E91D7-2180-489C-99F7-77346BAE4244}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="499" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="499" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Folha de salarios" sheetId="1" r:id="rId1"/>
@@ -1835,6 +1835,12 @@
     <xf numFmtId="17" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="15" fontId="36" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1844,17 +1850,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="36" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -2241,40 +2241,40 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:39" ht="27.75" x14ac:dyDescent="0.2">
-      <c r="A4" s="244" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="244"/>
-      <c r="C4" s="244"/>
-      <c r="D4" s="244"/>
-      <c r="E4" s="244"/>
-      <c r="F4" s="244"/>
-      <c r="G4" s="244"/>
-      <c r="H4" s="244"/>
-      <c r="I4" s="244"/>
-      <c r="J4" s="244"/>
-      <c r="K4" s="244"/>
-      <c r="L4" s="244"/>
-      <c r="M4" s="244"/>
-      <c r="N4" s="244"/>
-      <c r="O4" s="244"/>
-      <c r="P4" s="244"/>
-      <c r="Q4" s="244"/>
-      <c r="R4" s="244"/>
-      <c r="S4" s="244"/>
-      <c r="T4" s="244"/>
-      <c r="U4" s="244"/>
-      <c r="V4" s="244"/>
-      <c r="W4" s="244"/>
-      <c r="X4" s="244"/>
-      <c r="Y4" s="244"/>
-      <c r="Z4" s="244"/>
-      <c r="AA4" s="244"/>
-      <c r="AB4" s="244"/>
-      <c r="AC4" s="244"/>
-      <c r="AD4" s="244"/>
-      <c r="AE4" s="244"/>
-      <c r="AF4" s="244"/>
+      <c r="A4" s="246" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="246"/>
+      <c r="C4" s="246"/>
+      <c r="D4" s="246"/>
+      <c r="E4" s="246"/>
+      <c r="F4" s="246"/>
+      <c r="G4" s="246"/>
+      <c r="H4" s="246"/>
+      <c r="I4" s="246"/>
+      <c r="J4" s="246"/>
+      <c r="K4" s="246"/>
+      <c r="L4" s="246"/>
+      <c r="M4" s="246"/>
+      <c r="N4" s="246"/>
+      <c r="O4" s="246"/>
+      <c r="P4" s="246"/>
+      <c r="Q4" s="246"/>
+      <c r="R4" s="246"/>
+      <c r="S4" s="246"/>
+      <c r="T4" s="246"/>
+      <c r="U4" s="246"/>
+      <c r="V4" s="246"/>
+      <c r="W4" s="246"/>
+      <c r="X4" s="246"/>
+      <c r="Y4" s="246"/>
+      <c r="Z4" s="246"/>
+      <c r="AA4" s="246"/>
+      <c r="AB4" s="246"/>
+      <c r="AC4" s="246"/>
+      <c r="AD4" s="246"/>
+      <c r="AE4" s="246"/>
+      <c r="AF4" s="246"/>
       <c r="AG4" s="4"/>
       <c r="AH4" s="15" t="s">
         <v>1</v>
@@ -2419,53 +2419,53 @@
       <c r="AI7" s="38"/>
     </row>
     <row r="8" spans="1:39" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="248" t="s">
+      <c r="A8" s="245" t="s">
         <v>11</v>
       </c>
       <c r="B8" s="148"/>
-      <c r="C8" s="248" t="s">
+      <c r="C8" s="245" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="247" t="s">
+      <c r="D8" s="244" t="s">
         <v>126</v>
       </c>
-      <c r="E8" s="247" t="s">
+      <c r="E8" s="244" t="s">
         <v>128</v>
       </c>
       <c r="F8" s="242"/>
-      <c r="G8" s="248" t="s">
+      <c r="G8" s="245" t="s">
         <v>127</v>
       </c>
-      <c r="H8" s="248" t="s">
+      <c r="H8" s="245" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="248" t="s">
+      <c r="I8" s="245" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="248"/>
-      <c r="K8" s="248"/>
-      <c r="L8" s="248"/>
-      <c r="M8" s="248"/>
-      <c r="N8" s="248"/>
-      <c r="O8" s="248"/>
-      <c r="P8" s="248"/>
-      <c r="Q8" s="248"/>
-      <c r="R8" s="248"/>
-      <c r="S8" s="248"/>
-      <c r="T8" s="248"/>
-      <c r="U8" s="248"/>
-      <c r="V8" s="248"/>
-      <c r="W8" s="248"/>
-      <c r="X8" s="248"/>
-      <c r="Y8" s="248"/>
+      <c r="J8" s="245"/>
+      <c r="K8" s="245"/>
+      <c r="L8" s="245"/>
+      <c r="M8" s="245"/>
+      <c r="N8" s="245"/>
+      <c r="O8" s="245"/>
+      <c r="P8" s="245"/>
+      <c r="Q8" s="245"/>
+      <c r="R8" s="245"/>
+      <c r="S8" s="245"/>
+      <c r="T8" s="245"/>
+      <c r="U8" s="245"/>
+      <c r="V8" s="245"/>
+      <c r="W8" s="245"/>
+      <c r="X8" s="245"/>
+      <c r="Y8" s="245"/>
       <c r="Z8" s="148"/>
-      <c r="AA8" s="248" t="s">
+      <c r="AA8" s="245" t="s">
         <v>15</v>
       </c>
-      <c r="AB8" s="248"/>
-      <c r="AC8" s="248"/>
-      <c r="AD8" s="248"/>
-      <c r="AE8" s="248"/>
+      <c r="AB8" s="245"/>
+      <c r="AC8" s="245"/>
+      <c r="AD8" s="245"/>
+      <c r="AE8" s="245"/>
       <c r="AF8" s="149"/>
       <c r="AG8" s="150"/>
       <c r="AH8" s="149"/>
@@ -2475,16 +2475,16 @@
       <c r="AL8" s="14"/>
     </row>
     <row r="9" spans="1:39" s="6" customFormat="1" ht="279.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="248"/>
+      <c r="A9" s="245"/>
       <c r="B9" s="148"/>
-      <c r="C9" s="248"/>
-      <c r="D9" s="247"/>
-      <c r="E9" s="247"/>
+      <c r="C9" s="245"/>
+      <c r="D9" s="244"/>
+      <c r="E9" s="244"/>
       <c r="F9" s="242" t="s">
         <v>131</v>
       </c>
-      <c r="G9" s="248"/>
-      <c r="H9" s="248"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
       <c r="I9" s="151" t="s">
         <v>124</v>
       </c>
@@ -2560,7 +2560,7 @@
       <c r="AG9" s="158" t="s">
         <v>35</v>
       </c>
-      <c r="AH9" s="149" t="s">
+      <c r="AH9" s="158" t="s">
         <v>36</v>
       </c>
       <c r="AI9" s="240"/>
@@ -5559,16 +5559,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:155" ht="27.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="244" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="244"/>
-      <c r="C1" s="244"/>
-      <c r="D1" s="244"/>
-      <c r="E1" s="244"/>
-      <c r="F1" s="244"/>
-      <c r="G1" s="244"/>
-      <c r="H1" s="244"/>
+      <c r="A1" s="246" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="246"/>
+      <c r="C1" s="246"/>
+      <c r="D1" s="246"/>
+      <c r="E1" s="246"/>
+      <c r="F1" s="246"/>
+      <c r="G1" s="246"/>
+      <c r="H1" s="246"/>
       <c r="I1" s="4"/>
       <c r="J1" s="15" t="s">
         <v>1</v>
@@ -5619,18 +5619,18 @@
       <c r="J4" s="38"/>
     </row>
     <row r="5" spans="1:155" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="245" t="s">
+      <c r="A5" s="247" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="3"/>
-      <c r="C5" s="245" t="s">
+      <c r="C5" s="247" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="3"/>
-      <c r="E5" s="245"/>
-      <c r="F5" s="245"/>
+      <c r="E5" s="247"/>
+      <c r="F5" s="247"/>
       <c r="G5" s="39"/>
-      <c r="H5" s="246" t="s">
+      <c r="H5" s="248" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="2"/>
@@ -5640,9 +5640,9 @@
       <c r="M5" s="14"/>
     </row>
     <row r="6" spans="1:155" s="6" customFormat="1" ht="279.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="245"/>
+      <c r="A6" s="247"/>
       <c r="B6" s="3"/>
-      <c r="C6" s="245"/>
+      <c r="C6" s="247"/>
       <c r="D6" s="39" t="s">
         <v>29</v>
       </c>
@@ -5655,7 +5655,7 @@
       <c r="G6" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="246"/>
+      <c r="H6" s="248"/>
       <c r="I6" s="2"/>
       <c r="J6" s="39" t="s">
         <v>36</v>
@@ -7226,24 +7226,24 @@
   <sheetData>
     <row r="1" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="125"/>
-      <c r="B1" s="249" t="s">
+      <c r="B1" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="249"/>
-      <c r="D1" s="249"/>
-      <c r="E1" s="249"/>
-      <c r="F1" s="249"/>
-      <c r="G1" s="249"/>
+      <c r="C1" s="250"/>
+      <c r="D1" s="250"/>
+      <c r="E1" s="250"/>
+      <c r="F1" s="250"/>
+      <c r="G1" s="250"/>
       <c r="H1" s="127"/>
       <c r="I1" s="127"/>
-      <c r="J1" s="249" t="s">
+      <c r="J1" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K1" s="249"/>
-      <c r="L1" s="249"/>
-      <c r="M1" s="249"/>
-      <c r="N1" s="249"/>
-      <c r="O1" s="249"/>
+      <c r="K1" s="250"/>
+      <c r="L1" s="250"/>
+      <c r="M1" s="250"/>
+      <c r="N1" s="250"/>
+      <c r="O1" s="250"/>
     </row>
     <row r="2" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="125"/>
@@ -7264,24 +7264,24 @@
     </row>
     <row r="3" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="125"/>
-      <c r="B3" s="250" t="s">
+      <c r="B3" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="250"/>
-      <c r="D3" s="250"/>
-      <c r="E3" s="250"/>
-      <c r="F3" s="250"/>
-      <c r="G3" s="250"/>
+      <c r="C3" s="249"/>
+      <c r="D3" s="249"/>
+      <c r="E3" s="249"/>
+      <c r="F3" s="249"/>
+      <c r="G3" s="249"/>
       <c r="H3" s="129"/>
       <c r="I3" s="130"/>
-      <c r="J3" s="250" t="s">
+      <c r="J3" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K3" s="250"/>
-      <c r="L3" s="250"/>
-      <c r="M3" s="250"/>
-      <c r="N3" s="250"/>
-      <c r="O3" s="250"/>
+      <c r="K3" s="249"/>
+      <c r="L3" s="249"/>
+      <c r="M3" s="249"/>
+      <c r="N3" s="249"/>
+      <c r="O3" s="249"/>
     </row>
     <row r="4" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="125"/>
@@ -7889,24 +7889,24 @@
     </row>
     <row r="30" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="125"/>
-      <c r="B30" s="249" t="s">
+      <c r="B30" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="249"/>
-      <c r="D30" s="249"/>
-      <c r="E30" s="249"/>
-      <c r="F30" s="249"/>
-      <c r="G30" s="249"/>
+      <c r="C30" s="250"/>
+      <c r="D30" s="250"/>
+      <c r="E30" s="250"/>
+      <c r="F30" s="250"/>
+      <c r="G30" s="250"/>
       <c r="H30" s="127"/>
       <c r="I30" s="127"/>
-      <c r="J30" s="249" t="s">
+      <c r="J30" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K30" s="249"/>
-      <c r="L30" s="249"/>
-      <c r="M30" s="249"/>
-      <c r="N30" s="249"/>
-      <c r="O30" s="249"/>
+      <c r="K30" s="250"/>
+      <c r="L30" s="250"/>
+      <c r="M30" s="250"/>
+      <c r="N30" s="250"/>
+      <c r="O30" s="250"/>
     </row>
     <row r="31" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="125"/>
@@ -7927,24 +7927,24 @@
     </row>
     <row r="32" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="125"/>
-      <c r="B32" s="250" t="s">
+      <c r="B32" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C32" s="250"/>
-      <c r="D32" s="250"/>
-      <c r="E32" s="250"/>
-      <c r="F32" s="250"/>
-      <c r="G32" s="250"/>
+      <c r="C32" s="249"/>
+      <c r="D32" s="249"/>
+      <c r="E32" s="249"/>
+      <c r="F32" s="249"/>
+      <c r="G32" s="249"/>
       <c r="H32" s="129"/>
       <c r="I32" s="130"/>
-      <c r="J32" s="250" t="s">
+      <c r="J32" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K32" s="250"/>
-      <c r="L32" s="250"/>
-      <c r="M32" s="250"/>
-      <c r="N32" s="250"/>
-      <c r="O32" s="250"/>
+      <c r="K32" s="249"/>
+      <c r="L32" s="249"/>
+      <c r="M32" s="249"/>
+      <c r="N32" s="249"/>
+      <c r="O32" s="249"/>
     </row>
     <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="125"/>
@@ -8559,24 +8559,24 @@
     </row>
     <row r="59" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="125"/>
-      <c r="B59" s="249" t="s">
+      <c r="B59" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C59" s="249"/>
-      <c r="D59" s="249"/>
-      <c r="E59" s="249"/>
-      <c r="F59" s="249"/>
-      <c r="G59" s="249"/>
+      <c r="C59" s="250"/>
+      <c r="D59" s="250"/>
+      <c r="E59" s="250"/>
+      <c r="F59" s="250"/>
+      <c r="G59" s="250"/>
       <c r="H59" s="127"/>
       <c r="I59" s="127"/>
-      <c r="J59" s="249" t="s">
+      <c r="J59" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K59" s="249"/>
-      <c r="L59" s="249"/>
-      <c r="M59" s="249"/>
-      <c r="N59" s="249"/>
-      <c r="O59" s="249"/>
+      <c r="K59" s="250"/>
+      <c r="L59" s="250"/>
+      <c r="M59" s="250"/>
+      <c r="N59" s="250"/>
+      <c r="O59" s="250"/>
     </row>
     <row r="60" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="125"/>
@@ -8597,24 +8597,24 @@
     </row>
     <row r="61" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="125"/>
-      <c r="B61" s="250" t="s">
+      <c r="B61" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C61" s="250"/>
-      <c r="D61" s="250"/>
-      <c r="E61" s="250"/>
-      <c r="F61" s="250"/>
-      <c r="G61" s="250"/>
+      <c r="C61" s="249"/>
+      <c r="D61" s="249"/>
+      <c r="E61" s="249"/>
+      <c r="F61" s="249"/>
+      <c r="G61" s="249"/>
       <c r="H61" s="129"/>
       <c r="I61" s="130"/>
-      <c r="J61" s="250" t="s">
+      <c r="J61" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K61" s="250"/>
-      <c r="L61" s="250"/>
-      <c r="M61" s="250"/>
-      <c r="N61" s="250"/>
-      <c r="O61" s="250"/>
+      <c r="K61" s="249"/>
+      <c r="L61" s="249"/>
+      <c r="M61" s="249"/>
+      <c r="N61" s="249"/>
+      <c r="O61" s="249"/>
     </row>
     <row r="62" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="125"/>
@@ -9227,24 +9227,24 @@
     </row>
     <row r="88" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="125"/>
-      <c r="B88" s="249" t="s">
+      <c r="B88" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C88" s="249"/>
-      <c r="D88" s="249"/>
-      <c r="E88" s="249"/>
-      <c r="F88" s="249"/>
-      <c r="G88" s="249"/>
+      <c r="C88" s="250"/>
+      <c r="D88" s="250"/>
+      <c r="E88" s="250"/>
+      <c r="F88" s="250"/>
+      <c r="G88" s="250"/>
       <c r="H88" s="127"/>
       <c r="I88" s="127"/>
-      <c r="J88" s="249" t="s">
+      <c r="J88" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K88" s="249"/>
-      <c r="L88" s="249"/>
-      <c r="M88" s="249"/>
-      <c r="N88" s="249"/>
-      <c r="O88" s="249"/>
+      <c r="K88" s="250"/>
+      <c r="L88" s="250"/>
+      <c r="M88" s="250"/>
+      <c r="N88" s="250"/>
+      <c r="O88" s="250"/>
     </row>
     <row r="89" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="125"/>
@@ -9265,24 +9265,24 @@
     </row>
     <row r="90" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="125"/>
-      <c r="B90" s="250" t="s">
+      <c r="B90" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C90" s="250"/>
-      <c r="D90" s="250"/>
-      <c r="E90" s="250"/>
-      <c r="F90" s="250"/>
-      <c r="G90" s="250"/>
+      <c r="C90" s="249"/>
+      <c r="D90" s="249"/>
+      <c r="E90" s="249"/>
+      <c r="F90" s="249"/>
+      <c r="G90" s="249"/>
       <c r="H90" s="129"/>
       <c r="I90" s="130"/>
-      <c r="J90" s="250" t="s">
+      <c r="J90" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K90" s="250"/>
-      <c r="L90" s="250"/>
-      <c r="M90" s="250"/>
-      <c r="N90" s="250"/>
-      <c r="O90" s="250"/>
+      <c r="K90" s="249"/>
+      <c r="L90" s="249"/>
+      <c r="M90" s="249"/>
+      <c r="N90" s="249"/>
+      <c r="O90" s="249"/>
     </row>
     <row r="91" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="125"/>
@@ -9881,24 +9881,24 @@
     </row>
     <row r="116" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="125"/>
-      <c r="B116" s="249" t="s">
+      <c r="B116" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C116" s="249"/>
-      <c r="D116" s="249"/>
-      <c r="E116" s="249"/>
-      <c r="F116" s="249"/>
-      <c r="G116" s="249"/>
+      <c r="C116" s="250"/>
+      <c r="D116" s="250"/>
+      <c r="E116" s="250"/>
+      <c r="F116" s="250"/>
+      <c r="G116" s="250"/>
       <c r="H116" s="127"/>
       <c r="I116" s="127"/>
-      <c r="J116" s="249" t="s">
+      <c r="J116" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K116" s="249"/>
-      <c r="L116" s="249"/>
-      <c r="M116" s="249"/>
-      <c r="N116" s="249"/>
-      <c r="O116" s="249"/>
+      <c r="K116" s="250"/>
+      <c r="L116" s="250"/>
+      <c r="M116" s="250"/>
+      <c r="N116" s="250"/>
+      <c r="O116" s="250"/>
     </row>
     <row r="117" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="125"/>
@@ -9919,24 +9919,24 @@
     </row>
     <row r="118" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="125"/>
-      <c r="B118" s="250" t="s">
+      <c r="B118" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C118" s="250"/>
-      <c r="D118" s="250"/>
-      <c r="E118" s="250"/>
-      <c r="F118" s="250"/>
-      <c r="G118" s="250"/>
+      <c r="C118" s="249"/>
+      <c r="D118" s="249"/>
+      <c r="E118" s="249"/>
+      <c r="F118" s="249"/>
+      <c r="G118" s="249"/>
       <c r="H118" s="129"/>
       <c r="I118" s="130"/>
-      <c r="J118" s="250" t="s">
+      <c r="J118" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K118" s="250"/>
-      <c r="L118" s="250"/>
-      <c r="M118" s="250"/>
-      <c r="N118" s="250"/>
-      <c r="O118" s="250"/>
+      <c r="K118" s="249"/>
+      <c r="L118" s="249"/>
+      <c r="M118" s="249"/>
+      <c r="N118" s="249"/>
+      <c r="O118" s="249"/>
     </row>
     <row r="119" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="125"/>
@@ -10553,24 +10553,24 @@
     </row>
     <row r="145" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="125"/>
-      <c r="B145" s="249" t="s">
+      <c r="B145" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C145" s="249"/>
-      <c r="D145" s="249"/>
-      <c r="E145" s="249"/>
-      <c r="F145" s="249"/>
-      <c r="G145" s="249"/>
+      <c r="C145" s="250"/>
+      <c r="D145" s="250"/>
+      <c r="E145" s="250"/>
+      <c r="F145" s="250"/>
+      <c r="G145" s="250"/>
       <c r="H145" s="127"/>
       <c r="I145" s="127"/>
-      <c r="J145" s="249" t="s">
+      <c r="J145" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K145" s="249"/>
-      <c r="L145" s="249"/>
-      <c r="M145" s="249"/>
-      <c r="N145" s="249"/>
-      <c r="O145" s="249"/>
+      <c r="K145" s="250"/>
+      <c r="L145" s="250"/>
+      <c r="M145" s="250"/>
+      <c r="N145" s="250"/>
+      <c r="O145" s="250"/>
     </row>
     <row r="146" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="125"/>
@@ -10591,24 +10591,24 @@
     </row>
     <row r="147" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="125"/>
-      <c r="B147" s="250" t="s">
+      <c r="B147" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C147" s="250"/>
-      <c r="D147" s="250"/>
-      <c r="E147" s="250"/>
-      <c r="F147" s="250"/>
-      <c r="G147" s="250"/>
+      <c r="C147" s="249"/>
+      <c r="D147" s="249"/>
+      <c r="E147" s="249"/>
+      <c r="F147" s="249"/>
+      <c r="G147" s="249"/>
       <c r="H147" s="129"/>
       <c r="I147" s="130"/>
-      <c r="J147" s="250" t="s">
+      <c r="J147" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K147" s="250"/>
-      <c r="L147" s="250"/>
-      <c r="M147" s="250"/>
-      <c r="N147" s="250"/>
-      <c r="O147" s="250"/>
+      <c r="K147" s="249"/>
+      <c r="L147" s="249"/>
+      <c r="M147" s="249"/>
+      <c r="N147" s="249"/>
+      <c r="O147" s="249"/>
     </row>
     <row r="148" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="125"/>
@@ -11204,24 +11204,24 @@
     </row>
     <row r="173" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="125"/>
-      <c r="B173" s="249" t="s">
+      <c r="B173" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C173" s="249"/>
-      <c r="D173" s="249"/>
-      <c r="E173" s="249"/>
-      <c r="F173" s="249"/>
-      <c r="G173" s="249"/>
+      <c r="C173" s="250"/>
+      <c r="D173" s="250"/>
+      <c r="E173" s="250"/>
+      <c r="F173" s="250"/>
+      <c r="G173" s="250"/>
       <c r="H173" s="127"/>
       <c r="I173" s="127"/>
-      <c r="J173" s="249" t="s">
+      <c r="J173" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K173" s="249"/>
-      <c r="L173" s="249"/>
-      <c r="M173" s="249"/>
-      <c r="N173" s="249"/>
-      <c r="O173" s="249"/>
+      <c r="K173" s="250"/>
+      <c r="L173" s="250"/>
+      <c r="M173" s="250"/>
+      <c r="N173" s="250"/>
+      <c r="O173" s="250"/>
     </row>
     <row r="174" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="125"/>
@@ -11242,24 +11242,24 @@
     </row>
     <row r="175" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="125"/>
-      <c r="B175" s="250" t="s">
+      <c r="B175" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C175" s="250"/>
-      <c r="D175" s="250"/>
-      <c r="E175" s="250"/>
-      <c r="F175" s="250"/>
-      <c r="G175" s="250"/>
+      <c r="C175" s="249"/>
+      <c r="D175" s="249"/>
+      <c r="E175" s="249"/>
+      <c r="F175" s="249"/>
+      <c r="G175" s="249"/>
       <c r="H175" s="129"/>
       <c r="I175" s="130"/>
-      <c r="J175" s="250" t="s">
+      <c r="J175" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K175" s="250"/>
-      <c r="L175" s="250"/>
-      <c r="M175" s="250"/>
-      <c r="N175" s="250"/>
-      <c r="O175" s="250"/>
+      <c r="K175" s="249"/>
+      <c r="L175" s="249"/>
+      <c r="M175" s="249"/>
+      <c r="N175" s="249"/>
+      <c r="O175" s="249"/>
     </row>
     <row r="176" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="125"/>
@@ -11880,24 +11880,24 @@
     </row>
     <row r="202" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202" s="125"/>
-      <c r="B202" s="249" t="s">
+      <c r="B202" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C202" s="249"/>
-      <c r="D202" s="249"/>
-      <c r="E202" s="249"/>
-      <c r="F202" s="249"/>
-      <c r="G202" s="249"/>
+      <c r="C202" s="250"/>
+      <c r="D202" s="250"/>
+      <c r="E202" s="250"/>
+      <c r="F202" s="250"/>
+      <c r="G202" s="250"/>
       <c r="H202" s="127"/>
       <c r="I202" s="127"/>
-      <c r="J202" s="249" t="s">
+      <c r="J202" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K202" s="249"/>
-      <c r="L202" s="249"/>
-      <c r="M202" s="249"/>
-      <c r="N202" s="249"/>
-      <c r="O202" s="249"/>
+      <c r="K202" s="250"/>
+      <c r="L202" s="250"/>
+      <c r="M202" s="250"/>
+      <c r="N202" s="250"/>
+      <c r="O202" s="250"/>
     </row>
     <row r="203" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203" s="125"/>
@@ -11918,24 +11918,24 @@
     </row>
     <row r="204" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="125"/>
-      <c r="B204" s="250" t="s">
+      <c r="B204" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C204" s="250"/>
-      <c r="D204" s="250"/>
-      <c r="E204" s="250"/>
-      <c r="F204" s="250"/>
-      <c r="G204" s="250"/>
+      <c r="C204" s="249"/>
+      <c r="D204" s="249"/>
+      <c r="E204" s="249"/>
+      <c r="F204" s="249"/>
+      <c r="G204" s="249"/>
       <c r="H204" s="129"/>
       <c r="I204" s="130"/>
-      <c r="J204" s="250" t="s">
+      <c r="J204" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K204" s="250"/>
-      <c r="L204" s="250"/>
-      <c r="M204" s="250"/>
-      <c r="N204" s="250"/>
-      <c r="O204" s="250"/>
+      <c r="K204" s="249"/>
+      <c r="L204" s="249"/>
+      <c r="M204" s="249"/>
+      <c r="N204" s="249"/>
+      <c r="O204" s="249"/>
     </row>
     <row r="205" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="125"/>
@@ -12556,24 +12556,24 @@
     </row>
     <row r="231" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="125"/>
-      <c r="B231" s="249" t="s">
+      <c r="B231" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C231" s="249"/>
-      <c r="D231" s="249"/>
-      <c r="E231" s="249"/>
-      <c r="F231" s="249"/>
-      <c r="G231" s="249"/>
+      <c r="C231" s="250"/>
+      <c r="D231" s="250"/>
+      <c r="E231" s="250"/>
+      <c r="F231" s="250"/>
+      <c r="G231" s="250"/>
       <c r="H231" s="127"/>
       <c r="I231" s="127"/>
-      <c r="J231" s="249" t="s">
+      <c r="J231" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K231" s="249"/>
-      <c r="L231" s="249"/>
-      <c r="M231" s="249"/>
-      <c r="N231" s="249"/>
-      <c r="O231" s="249"/>
+      <c r="K231" s="250"/>
+      <c r="L231" s="250"/>
+      <c r="M231" s="250"/>
+      <c r="N231" s="250"/>
+      <c r="O231" s="250"/>
     </row>
     <row r="232" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232" s="125"/>
@@ -12594,24 +12594,24 @@
     </row>
     <row r="233" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="125"/>
-      <c r="B233" s="250" t="s">
+      <c r="B233" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C233" s="250"/>
-      <c r="D233" s="250"/>
-      <c r="E233" s="250"/>
-      <c r="F233" s="250"/>
-      <c r="G233" s="250"/>
+      <c r="C233" s="249"/>
+      <c r="D233" s="249"/>
+      <c r="E233" s="249"/>
+      <c r="F233" s="249"/>
+      <c r="G233" s="249"/>
       <c r="H233" s="129"/>
       <c r="I233" s="130"/>
-      <c r="J233" s="250" t="s">
+      <c r="J233" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K233" s="250"/>
-      <c r="L233" s="250"/>
-      <c r="M233" s="250"/>
-      <c r="N233" s="250"/>
-      <c r="O233" s="250"/>
+      <c r="K233" s="249"/>
+      <c r="L233" s="249"/>
+      <c r="M233" s="249"/>
+      <c r="N233" s="249"/>
+      <c r="O233" s="249"/>
     </row>
     <row r="234" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234" s="125"/>
@@ -13233,24 +13233,24 @@
     </row>
     <row r="260" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="125"/>
-      <c r="B260" s="249" t="s">
+      <c r="B260" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C260" s="249"/>
-      <c r="D260" s="249"/>
-      <c r="E260" s="249"/>
-      <c r="F260" s="249"/>
-      <c r="G260" s="249"/>
+      <c r="C260" s="250"/>
+      <c r="D260" s="250"/>
+      <c r="E260" s="250"/>
+      <c r="F260" s="250"/>
+      <c r="G260" s="250"/>
       <c r="H260" s="127"/>
       <c r="I260" s="127"/>
-      <c r="J260" s="249" t="s">
+      <c r="J260" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K260" s="249"/>
-      <c r="L260" s="249"/>
-      <c r="M260" s="249"/>
-      <c r="N260" s="249"/>
-      <c r="O260" s="249"/>
+      <c r="K260" s="250"/>
+      <c r="L260" s="250"/>
+      <c r="M260" s="250"/>
+      <c r="N260" s="250"/>
+      <c r="O260" s="250"/>
     </row>
     <row r="261" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="125"/>
@@ -13271,24 +13271,24 @@
     </row>
     <row r="262" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A262" s="125"/>
-      <c r="B262" s="250" t="s">
+      <c r="B262" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C262" s="250"/>
-      <c r="D262" s="250"/>
-      <c r="E262" s="250"/>
-      <c r="F262" s="250"/>
-      <c r="G262" s="250"/>
+      <c r="C262" s="249"/>
+      <c r="D262" s="249"/>
+      <c r="E262" s="249"/>
+      <c r="F262" s="249"/>
+      <c r="G262" s="249"/>
       <c r="H262" s="129"/>
       <c r="I262" s="130"/>
-      <c r="J262" s="250" t="s">
+      <c r="J262" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K262" s="250"/>
-      <c r="L262" s="250"/>
-      <c r="M262" s="250"/>
-      <c r="N262" s="250"/>
-      <c r="O262" s="250"/>
+      <c r="K262" s="249"/>
+      <c r="L262" s="249"/>
+      <c r="M262" s="249"/>
+      <c r="N262" s="249"/>
+      <c r="O262" s="249"/>
     </row>
     <row r="263" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="125"/>
@@ -13912,24 +13912,24 @@
     </row>
     <row r="289" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289" s="125"/>
-      <c r="B289" s="249" t="s">
+      <c r="B289" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C289" s="249"/>
-      <c r="D289" s="249"/>
-      <c r="E289" s="249"/>
-      <c r="F289" s="249"/>
-      <c r="G289" s="249"/>
+      <c r="C289" s="250"/>
+      <c r="D289" s="250"/>
+      <c r="E289" s="250"/>
+      <c r="F289" s="250"/>
+      <c r="G289" s="250"/>
       <c r="H289" s="127"/>
       <c r="I289" s="127"/>
-      <c r="J289" s="249" t="s">
+      <c r="J289" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K289" s="249"/>
-      <c r="L289" s="249"/>
-      <c r="M289" s="249"/>
-      <c r="N289" s="249"/>
-      <c r="O289" s="249"/>
+      <c r="K289" s="250"/>
+      <c r="L289" s="250"/>
+      <c r="M289" s="250"/>
+      <c r="N289" s="250"/>
+      <c r="O289" s="250"/>
     </row>
     <row r="290" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A290" s="125"/>
@@ -13950,24 +13950,24 @@
     </row>
     <row r="291" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A291" s="125"/>
-      <c r="B291" s="250" t="s">
+      <c r="B291" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C291" s="250"/>
-      <c r="D291" s="250"/>
-      <c r="E291" s="250"/>
-      <c r="F291" s="250"/>
-      <c r="G291" s="250"/>
+      <c r="C291" s="249"/>
+      <c r="D291" s="249"/>
+      <c r="E291" s="249"/>
+      <c r="F291" s="249"/>
+      <c r="G291" s="249"/>
       <c r="H291" s="129"/>
       <c r="I291" s="130"/>
-      <c r="J291" s="250" t="s">
+      <c r="J291" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K291" s="250"/>
-      <c r="L291" s="250"/>
-      <c r="M291" s="250"/>
-      <c r="N291" s="250"/>
-      <c r="O291" s="250"/>
+      <c r="K291" s="249"/>
+      <c r="L291" s="249"/>
+      <c r="M291" s="249"/>
+      <c r="N291" s="249"/>
+      <c r="O291" s="249"/>
     </row>
     <row r="292" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A292" s="125"/>
@@ -14588,24 +14588,24 @@
     </row>
     <row r="318" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A318" s="125"/>
-      <c r="B318" s="249" t="s">
+      <c r="B318" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C318" s="249"/>
-      <c r="D318" s="249"/>
-      <c r="E318" s="249"/>
-      <c r="F318" s="249"/>
-      <c r="G318" s="249"/>
+      <c r="C318" s="250"/>
+      <c r="D318" s="250"/>
+      <c r="E318" s="250"/>
+      <c r="F318" s="250"/>
+      <c r="G318" s="250"/>
       <c r="H318" s="127"/>
       <c r="I318" s="127"/>
-      <c r="J318" s="249" t="s">
+      <c r="J318" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K318" s="249"/>
-      <c r="L318" s="249"/>
-      <c r="M318" s="249"/>
-      <c r="N318" s="249"/>
-      <c r="O318" s="249"/>
+      <c r="K318" s="250"/>
+      <c r="L318" s="250"/>
+      <c r="M318" s="250"/>
+      <c r="N318" s="250"/>
+      <c r="O318" s="250"/>
     </row>
     <row r="319" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A319" s="125"/>
@@ -14626,24 +14626,24 @@
     </row>
     <row r="320" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A320" s="125"/>
-      <c r="B320" s="250" t="s">
+      <c r="B320" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C320" s="250"/>
-      <c r="D320" s="250"/>
-      <c r="E320" s="250"/>
-      <c r="F320" s="250"/>
-      <c r="G320" s="250"/>
+      <c r="C320" s="249"/>
+      <c r="D320" s="249"/>
+      <c r="E320" s="249"/>
+      <c r="F320" s="249"/>
+      <c r="G320" s="249"/>
       <c r="H320" s="129"/>
       <c r="I320" s="130"/>
-      <c r="J320" s="250" t="s">
+      <c r="J320" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K320" s="250"/>
-      <c r="L320" s="250"/>
-      <c r="M320" s="250"/>
-      <c r="N320" s="250"/>
-      <c r="O320" s="250"/>
+      <c r="K320" s="249"/>
+      <c r="L320" s="249"/>
+      <c r="M320" s="249"/>
+      <c r="N320" s="249"/>
+      <c r="O320" s="249"/>
     </row>
     <row r="321" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A321" s="125"/>
@@ -15264,24 +15264,24 @@
     </row>
     <row r="347" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A347" s="125"/>
-      <c r="B347" s="249" t="s">
+      <c r="B347" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C347" s="249"/>
-      <c r="D347" s="249"/>
-      <c r="E347" s="249"/>
-      <c r="F347" s="249"/>
-      <c r="G347" s="249"/>
+      <c r="C347" s="250"/>
+      <c r="D347" s="250"/>
+      <c r="E347" s="250"/>
+      <c r="F347" s="250"/>
+      <c r="G347" s="250"/>
       <c r="H347" s="127"/>
       <c r="I347" s="127"/>
-      <c r="J347" s="249" t="s">
+      <c r="J347" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K347" s="249"/>
-      <c r="L347" s="249"/>
-      <c r="M347" s="249"/>
-      <c r="N347" s="249"/>
-      <c r="O347" s="249"/>
+      <c r="K347" s="250"/>
+      <c r="L347" s="250"/>
+      <c r="M347" s="250"/>
+      <c r="N347" s="250"/>
+      <c r="O347" s="250"/>
     </row>
     <row r="348" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A348" s="125"/>
@@ -15302,24 +15302,24 @@
     </row>
     <row r="349" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A349" s="125"/>
-      <c r="B349" s="250" t="s">
+      <c r="B349" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C349" s="250"/>
-      <c r="D349" s="250"/>
-      <c r="E349" s="250"/>
-      <c r="F349" s="250"/>
-      <c r="G349" s="250"/>
+      <c r="C349" s="249"/>
+      <c r="D349" s="249"/>
+      <c r="E349" s="249"/>
+      <c r="F349" s="249"/>
+      <c r="G349" s="249"/>
       <c r="H349" s="129"/>
       <c r="I349" s="130"/>
-      <c r="J349" s="250" t="s">
+      <c r="J349" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K349" s="250"/>
-      <c r="L349" s="250"/>
-      <c r="M349" s="250"/>
-      <c r="N349" s="250"/>
-      <c r="O349" s="250"/>
+      <c r="K349" s="249"/>
+      <c r="L349" s="249"/>
+      <c r="M349" s="249"/>
+      <c r="N349" s="249"/>
+      <c r="O349" s="249"/>
     </row>
     <row r="350" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A350" s="125"/>
@@ -15951,24 +15951,24 @@
     </row>
     <row r="376" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A376" s="125"/>
-      <c r="B376" s="249" t="s">
+      <c r="B376" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C376" s="249"/>
-      <c r="D376" s="249"/>
-      <c r="E376" s="249"/>
-      <c r="F376" s="249"/>
-      <c r="G376" s="249"/>
+      <c r="C376" s="250"/>
+      <c r="D376" s="250"/>
+      <c r="E376" s="250"/>
+      <c r="F376" s="250"/>
+      <c r="G376" s="250"/>
       <c r="H376" s="127"/>
       <c r="I376" s="127"/>
-      <c r="J376" s="249" t="s">
+      <c r="J376" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K376" s="249"/>
-      <c r="L376" s="249"/>
-      <c r="M376" s="249"/>
-      <c r="N376" s="249"/>
-      <c r="O376" s="249"/>
+      <c r="K376" s="250"/>
+      <c r="L376" s="250"/>
+      <c r="M376" s="250"/>
+      <c r="N376" s="250"/>
+      <c r="O376" s="250"/>
     </row>
     <row r="377" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A377" s="125"/>
@@ -15989,24 +15989,24 @@
     </row>
     <row r="378" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A378" s="125"/>
-      <c r="B378" s="250" t="s">
+      <c r="B378" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C378" s="250"/>
-      <c r="D378" s="250"/>
-      <c r="E378" s="250"/>
-      <c r="F378" s="250"/>
-      <c r="G378" s="250"/>
+      <c r="C378" s="249"/>
+      <c r="D378" s="249"/>
+      <c r="E378" s="249"/>
+      <c r="F378" s="249"/>
+      <c r="G378" s="249"/>
       <c r="H378" s="129"/>
       <c r="I378" s="130"/>
-      <c r="J378" s="250" t="s">
+      <c r="J378" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K378" s="250"/>
-      <c r="L378" s="250"/>
-      <c r="M378" s="250"/>
-      <c r="N378" s="250"/>
-      <c r="O378" s="250"/>
+      <c r="K378" s="249"/>
+      <c r="L378" s="249"/>
+      <c r="M378" s="249"/>
+      <c r="N378" s="249"/>
+      <c r="O378" s="249"/>
     </row>
     <row r="379" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A379" s="125"/>
@@ -16628,24 +16628,24 @@
     </row>
     <row r="405" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A405" s="125"/>
-      <c r="B405" s="249" t="s">
+      <c r="B405" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C405" s="249"/>
-      <c r="D405" s="249"/>
-      <c r="E405" s="249"/>
-      <c r="F405" s="249"/>
-      <c r="G405" s="249"/>
+      <c r="C405" s="250"/>
+      <c r="D405" s="250"/>
+      <c r="E405" s="250"/>
+      <c r="F405" s="250"/>
+      <c r="G405" s="250"/>
       <c r="H405" s="127"/>
       <c r="I405" s="127"/>
-      <c r="J405" s="249" t="s">
+      <c r="J405" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K405" s="249"/>
-      <c r="L405" s="249"/>
-      <c r="M405" s="249"/>
-      <c r="N405" s="249"/>
-      <c r="O405" s="249"/>
+      <c r="K405" s="250"/>
+      <c r="L405" s="250"/>
+      <c r="M405" s="250"/>
+      <c r="N405" s="250"/>
+      <c r="O405" s="250"/>
     </row>
     <row r="406" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A406" s="125"/>
@@ -16666,24 +16666,24 @@
     </row>
     <row r="407" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A407" s="125"/>
-      <c r="B407" s="250" t="s">
+      <c r="B407" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C407" s="250"/>
-      <c r="D407" s="250"/>
-      <c r="E407" s="250"/>
-      <c r="F407" s="250"/>
-      <c r="G407" s="250"/>
+      <c r="C407" s="249"/>
+      <c r="D407" s="249"/>
+      <c r="E407" s="249"/>
+      <c r="F407" s="249"/>
+      <c r="G407" s="249"/>
       <c r="H407" s="129"/>
       <c r="I407" s="130"/>
-      <c r="J407" s="250" t="s">
+      <c r="J407" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K407" s="250"/>
-      <c r="L407" s="250"/>
-      <c r="M407" s="250"/>
-      <c r="N407" s="250"/>
-      <c r="O407" s="250"/>
+      <c r="K407" s="249"/>
+      <c r="L407" s="249"/>
+      <c r="M407" s="249"/>
+      <c r="N407" s="249"/>
+      <c r="O407" s="249"/>
     </row>
     <row r="408" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A408" s="125"/>
@@ -17309,24 +17309,24 @@
     </row>
     <row r="434" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A434" s="125"/>
-      <c r="B434" s="249" t="s">
+      <c r="B434" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C434" s="249"/>
-      <c r="D434" s="249"/>
-      <c r="E434" s="249"/>
-      <c r="F434" s="249"/>
-      <c r="G434" s="249"/>
+      <c r="C434" s="250"/>
+      <c r="D434" s="250"/>
+      <c r="E434" s="250"/>
+      <c r="F434" s="250"/>
+      <c r="G434" s="250"/>
       <c r="H434" s="127"/>
       <c r="I434" s="127"/>
-      <c r="J434" s="249" t="s">
+      <c r="J434" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K434" s="249"/>
-      <c r="L434" s="249"/>
-      <c r="M434" s="249"/>
-      <c r="N434" s="249"/>
-      <c r="O434" s="249"/>
+      <c r="K434" s="250"/>
+      <c r="L434" s="250"/>
+      <c r="M434" s="250"/>
+      <c r="N434" s="250"/>
+      <c r="O434" s="250"/>
     </row>
     <row r="435" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A435" s="125"/>
@@ -17347,24 +17347,24 @@
     </row>
     <row r="436" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A436" s="125"/>
-      <c r="B436" s="250" t="s">
+      <c r="B436" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C436" s="250"/>
-      <c r="D436" s="250"/>
-      <c r="E436" s="250"/>
-      <c r="F436" s="250"/>
-      <c r="G436" s="250"/>
+      <c r="C436" s="249"/>
+      <c r="D436" s="249"/>
+      <c r="E436" s="249"/>
+      <c r="F436" s="249"/>
+      <c r="G436" s="249"/>
       <c r="H436" s="129"/>
       <c r="I436" s="130"/>
-      <c r="J436" s="250" t="s">
+      <c r="J436" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K436" s="250"/>
-      <c r="L436" s="250"/>
-      <c r="M436" s="250"/>
-      <c r="N436" s="250"/>
-      <c r="O436" s="250"/>
+      <c r="K436" s="249"/>
+      <c r="L436" s="249"/>
+      <c r="M436" s="249"/>
+      <c r="N436" s="249"/>
+      <c r="O436" s="249"/>
     </row>
     <row r="437" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A437" s="125"/>
@@ -17961,24 +17961,24 @@
     </row>
     <row r="462" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A462" s="125"/>
-      <c r="B462" s="249" t="s">
+      <c r="B462" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C462" s="249"/>
-      <c r="D462" s="249"/>
-      <c r="E462" s="249"/>
-      <c r="F462" s="249"/>
-      <c r="G462" s="249"/>
+      <c r="C462" s="250"/>
+      <c r="D462" s="250"/>
+      <c r="E462" s="250"/>
+      <c r="F462" s="250"/>
+      <c r="G462" s="250"/>
       <c r="H462" s="127"/>
       <c r="I462" s="127"/>
-      <c r="J462" s="249" t="s">
+      <c r="J462" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K462" s="249"/>
-      <c r="L462" s="249"/>
-      <c r="M462" s="249"/>
-      <c r="N462" s="249"/>
-      <c r="O462" s="249"/>
+      <c r="K462" s="250"/>
+      <c r="L462" s="250"/>
+      <c r="M462" s="250"/>
+      <c r="N462" s="250"/>
+      <c r="O462" s="250"/>
     </row>
     <row r="463" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A463" s="125"/>
@@ -17999,24 +17999,24 @@
     </row>
     <row r="464" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A464" s="125"/>
-      <c r="B464" s="250" t="s">
+      <c r="B464" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C464" s="250"/>
-      <c r="D464" s="250"/>
-      <c r="E464" s="250"/>
-      <c r="F464" s="250"/>
-      <c r="G464" s="250"/>
+      <c r="C464" s="249"/>
+      <c r="D464" s="249"/>
+      <c r="E464" s="249"/>
+      <c r="F464" s="249"/>
+      <c r="G464" s="249"/>
       <c r="H464" s="129"/>
       <c r="I464" s="130"/>
-      <c r="J464" s="250" t="s">
+      <c r="J464" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K464" s="250"/>
-      <c r="L464" s="250"/>
-      <c r="M464" s="250"/>
-      <c r="N464" s="250"/>
-      <c r="O464" s="250"/>
+      <c r="K464" s="249"/>
+      <c r="L464" s="249"/>
+      <c r="M464" s="249"/>
+      <c r="N464" s="249"/>
+      <c r="O464" s="249"/>
     </row>
     <row r="465" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A465" s="125"/>
@@ -18637,24 +18637,24 @@
     </row>
     <row r="491" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A491" s="125"/>
-      <c r="B491" s="249" t="s">
+      <c r="B491" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C491" s="249"/>
-      <c r="D491" s="249"/>
-      <c r="E491" s="249"/>
-      <c r="F491" s="249"/>
-      <c r="G491" s="249"/>
+      <c r="C491" s="250"/>
+      <c r="D491" s="250"/>
+      <c r="E491" s="250"/>
+      <c r="F491" s="250"/>
+      <c r="G491" s="250"/>
       <c r="H491" s="127"/>
       <c r="I491" s="127"/>
-      <c r="J491" s="249" t="s">
+      <c r="J491" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K491" s="249"/>
-      <c r="L491" s="249"/>
-      <c r="M491" s="249"/>
-      <c r="N491" s="249"/>
-      <c r="O491" s="249"/>
+      <c r="K491" s="250"/>
+      <c r="L491" s="250"/>
+      <c r="M491" s="250"/>
+      <c r="N491" s="250"/>
+      <c r="O491" s="250"/>
     </row>
     <row r="492" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A492" s="125"/>
@@ -18675,24 +18675,24 @@
     </row>
     <row r="493" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A493" s="125"/>
-      <c r="B493" s="250" t="s">
+      <c r="B493" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C493" s="250"/>
-      <c r="D493" s="250"/>
-      <c r="E493" s="250"/>
-      <c r="F493" s="250"/>
-      <c r="G493" s="250"/>
+      <c r="C493" s="249"/>
+      <c r="D493" s="249"/>
+      <c r="E493" s="249"/>
+      <c r="F493" s="249"/>
+      <c r="G493" s="249"/>
       <c r="H493" s="129"/>
       <c r="I493" s="130"/>
-      <c r="J493" s="250" t="s">
+      <c r="J493" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K493" s="250"/>
-      <c r="L493" s="250"/>
-      <c r="M493" s="250"/>
-      <c r="N493" s="250"/>
-      <c r="O493" s="250"/>
+      <c r="K493" s="249"/>
+      <c r="L493" s="249"/>
+      <c r="M493" s="249"/>
+      <c r="N493" s="249"/>
+      <c r="O493" s="249"/>
     </row>
     <row r="494" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A494" s="125"/>
@@ -19315,24 +19315,24 @@
     </row>
     <row r="520" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A520" s="125"/>
-      <c r="B520" s="249" t="s">
+      <c r="B520" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C520" s="249"/>
-      <c r="D520" s="249"/>
-      <c r="E520" s="249"/>
-      <c r="F520" s="249"/>
-      <c r="G520" s="249"/>
+      <c r="C520" s="250"/>
+      <c r="D520" s="250"/>
+      <c r="E520" s="250"/>
+      <c r="F520" s="250"/>
+      <c r="G520" s="250"/>
       <c r="H520" s="127"/>
       <c r="I520" s="127"/>
-      <c r="J520" s="249" t="s">
+      <c r="J520" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K520" s="249"/>
-      <c r="L520" s="249"/>
-      <c r="M520" s="249"/>
-      <c r="N520" s="249"/>
-      <c r="O520" s="249"/>
+      <c r="K520" s="250"/>
+      <c r="L520" s="250"/>
+      <c r="M520" s="250"/>
+      <c r="N520" s="250"/>
+      <c r="O520" s="250"/>
     </row>
     <row r="521" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A521" s="125"/>
@@ -19353,24 +19353,24 @@
     </row>
     <row r="522" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A522" s="125"/>
-      <c r="B522" s="250" t="s">
+      <c r="B522" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C522" s="250"/>
-      <c r="D522" s="250"/>
-      <c r="E522" s="250"/>
-      <c r="F522" s="250"/>
-      <c r="G522" s="250"/>
+      <c r="C522" s="249"/>
+      <c r="D522" s="249"/>
+      <c r="E522" s="249"/>
+      <c r="F522" s="249"/>
+      <c r="G522" s="249"/>
       <c r="H522" s="129"/>
       <c r="I522" s="130"/>
-      <c r="J522" s="250" t="s">
+      <c r="J522" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K522" s="250"/>
-      <c r="L522" s="250"/>
-      <c r="M522" s="250"/>
-      <c r="N522" s="250"/>
-      <c r="O522" s="250"/>
+      <c r="K522" s="249"/>
+      <c r="L522" s="249"/>
+      <c r="M522" s="249"/>
+      <c r="N522" s="249"/>
+      <c r="O522" s="249"/>
     </row>
     <row r="523" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A523" s="125"/>
@@ -19993,24 +19993,24 @@
     </row>
     <row r="549" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A549" s="125"/>
-      <c r="B549" s="249" t="s">
+      <c r="B549" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C549" s="249"/>
-      <c r="D549" s="249"/>
-      <c r="E549" s="249"/>
-      <c r="F549" s="249"/>
-      <c r="G549" s="249"/>
+      <c r="C549" s="250"/>
+      <c r="D549" s="250"/>
+      <c r="E549" s="250"/>
+      <c r="F549" s="250"/>
+      <c r="G549" s="250"/>
       <c r="H549" s="127"/>
       <c r="I549" s="127"/>
-      <c r="J549" s="249" t="s">
+      <c r="J549" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K549" s="249"/>
-      <c r="L549" s="249"/>
-      <c r="M549" s="249"/>
-      <c r="N549" s="249"/>
-      <c r="O549" s="249"/>
+      <c r="K549" s="250"/>
+      <c r="L549" s="250"/>
+      <c r="M549" s="250"/>
+      <c r="N549" s="250"/>
+      <c r="O549" s="250"/>
     </row>
     <row r="550" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A550" s="125"/>
@@ -20031,24 +20031,24 @@
     </row>
     <row r="551" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A551" s="125"/>
-      <c r="B551" s="250" t="s">
+      <c r="B551" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C551" s="250"/>
-      <c r="D551" s="250"/>
-      <c r="E551" s="250"/>
-      <c r="F551" s="250"/>
-      <c r="G551" s="250"/>
+      <c r="C551" s="249"/>
+      <c r="D551" s="249"/>
+      <c r="E551" s="249"/>
+      <c r="F551" s="249"/>
+      <c r="G551" s="249"/>
       <c r="H551" s="129"/>
       <c r="I551" s="130"/>
-      <c r="J551" s="250" t="s">
+      <c r="J551" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K551" s="250"/>
-      <c r="L551" s="250"/>
-      <c r="M551" s="250"/>
-      <c r="N551" s="250"/>
-      <c r="O551" s="250"/>
+      <c r="K551" s="249"/>
+      <c r="L551" s="249"/>
+      <c r="M551" s="249"/>
+      <c r="N551" s="249"/>
+      <c r="O551" s="249"/>
     </row>
     <row r="552" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A552" s="125"/>
@@ -20671,24 +20671,24 @@
     </row>
     <row r="578" spans="1:15" ht="38.1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A578" s="125"/>
-      <c r="B578" s="249" t="s">
+      <c r="B578" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="C578" s="249"/>
-      <c r="D578" s="249"/>
-      <c r="E578" s="249"/>
-      <c r="F578" s="249"/>
-      <c r="G578" s="249"/>
+      <c r="C578" s="250"/>
+      <c r="D578" s="250"/>
+      <c r="E578" s="250"/>
+      <c r="F578" s="250"/>
+      <c r="G578" s="250"/>
       <c r="H578" s="127"/>
       <c r="I578" s="127"/>
-      <c r="J578" s="249" t="s">
+      <c r="J578" s="250" t="s">
         <v>91</v>
       </c>
-      <c r="K578" s="249"/>
-      <c r="L578" s="249"/>
-      <c r="M578" s="249"/>
-      <c r="N578" s="249"/>
-      <c r="O578" s="249"/>
+      <c r="K578" s="250"/>
+      <c r="L578" s="250"/>
+      <c r="M578" s="250"/>
+      <c r="N578" s="250"/>
+      <c r="O578" s="250"/>
     </row>
     <row r="579" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A579" s="125"/>
@@ -20709,24 +20709,24 @@
     </row>
     <row r="580" spans="1:15" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A580" s="125"/>
-      <c r="B580" s="250" t="s">
+      <c r="B580" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="C580" s="250"/>
-      <c r="D580" s="250"/>
-      <c r="E580" s="250"/>
-      <c r="F580" s="250"/>
-      <c r="G580" s="250"/>
+      <c r="C580" s="249"/>
+      <c r="D580" s="249"/>
+      <c r="E580" s="249"/>
+      <c r="F580" s="249"/>
+      <c r="G580" s="249"/>
       <c r="H580" s="129"/>
       <c r="I580" s="130"/>
-      <c r="J580" s="250" t="s">
+      <c r="J580" s="249" t="s">
         <v>92</v>
       </c>
-      <c r="K580" s="250"/>
-      <c r="L580" s="250"/>
-      <c r="M580" s="250"/>
-      <c r="N580" s="250"/>
-      <c r="O580" s="250"/>
+      <c r="K580" s="249"/>
+      <c r="L580" s="249"/>
+      <c r="M580" s="249"/>
+      <c r="N580" s="249"/>
+      <c r="O580" s="249"/>
     </row>
     <row r="581" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A581" s="125"/>
@@ -21400,74 +21400,6 @@
     </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="B522:G522"/>
-    <mergeCell ref="J522:O522"/>
-    <mergeCell ref="B549:G549"/>
-    <mergeCell ref="J549:O549"/>
-    <mergeCell ref="B551:G551"/>
-    <mergeCell ref="J551:O551"/>
-    <mergeCell ref="B520:G520"/>
-    <mergeCell ref="J520:O520"/>
-    <mergeCell ref="B493:G493"/>
-    <mergeCell ref="J493:O493"/>
-    <mergeCell ref="B462:G462"/>
-    <mergeCell ref="J462:O462"/>
-    <mergeCell ref="B464:G464"/>
-    <mergeCell ref="J464:O464"/>
-    <mergeCell ref="B491:G491"/>
-    <mergeCell ref="J491:O491"/>
-    <mergeCell ref="B434:G434"/>
-    <mergeCell ref="J434:O434"/>
-    <mergeCell ref="B436:G436"/>
-    <mergeCell ref="J436:O436"/>
-    <mergeCell ref="B376:G376"/>
-    <mergeCell ref="J376:O376"/>
-    <mergeCell ref="B378:G378"/>
-    <mergeCell ref="J378:O378"/>
-    <mergeCell ref="B405:G405"/>
-    <mergeCell ref="J405:O405"/>
-    <mergeCell ref="B407:G407"/>
-    <mergeCell ref="J407:O407"/>
-    <mergeCell ref="B320:G320"/>
-    <mergeCell ref="J320:O320"/>
-    <mergeCell ref="B347:G347"/>
-    <mergeCell ref="J347:O347"/>
-    <mergeCell ref="B349:G349"/>
-    <mergeCell ref="J349:O349"/>
-    <mergeCell ref="B289:G289"/>
-    <mergeCell ref="J289:O289"/>
-    <mergeCell ref="B291:G291"/>
-    <mergeCell ref="J291:O291"/>
-    <mergeCell ref="B318:G318"/>
-    <mergeCell ref="J318:O318"/>
-    <mergeCell ref="B233:G233"/>
-    <mergeCell ref="J233:O233"/>
-    <mergeCell ref="B260:G260"/>
-    <mergeCell ref="J260:O260"/>
-    <mergeCell ref="B262:G262"/>
-    <mergeCell ref="J262:O262"/>
-    <mergeCell ref="B173:G173"/>
-    <mergeCell ref="J173:O173"/>
-    <mergeCell ref="B175:G175"/>
-    <mergeCell ref="J175:O175"/>
-    <mergeCell ref="B231:G231"/>
-    <mergeCell ref="J231:O231"/>
-    <mergeCell ref="B202:G202"/>
-    <mergeCell ref="J202:O202"/>
-    <mergeCell ref="B204:G204"/>
-    <mergeCell ref="J204:O204"/>
-    <mergeCell ref="B118:G118"/>
-    <mergeCell ref="J118:O118"/>
-    <mergeCell ref="B145:G145"/>
-    <mergeCell ref="J145:O145"/>
-    <mergeCell ref="B147:G147"/>
-    <mergeCell ref="J147:O147"/>
-    <mergeCell ref="B88:G88"/>
-    <mergeCell ref="J88:O88"/>
-    <mergeCell ref="B90:G90"/>
-    <mergeCell ref="J90:O90"/>
-    <mergeCell ref="B116:G116"/>
-    <mergeCell ref="J116:O116"/>
     <mergeCell ref="B578:G578"/>
     <mergeCell ref="J578:O578"/>
     <mergeCell ref="B580:G580"/>
@@ -21484,6 +21416,74 @@
     <mergeCell ref="J59:O59"/>
     <mergeCell ref="B61:G61"/>
     <mergeCell ref="J61:O61"/>
+    <mergeCell ref="B88:G88"/>
+    <mergeCell ref="J88:O88"/>
+    <mergeCell ref="B90:G90"/>
+    <mergeCell ref="J90:O90"/>
+    <mergeCell ref="B116:G116"/>
+    <mergeCell ref="J116:O116"/>
+    <mergeCell ref="B118:G118"/>
+    <mergeCell ref="J118:O118"/>
+    <mergeCell ref="B145:G145"/>
+    <mergeCell ref="J145:O145"/>
+    <mergeCell ref="B147:G147"/>
+    <mergeCell ref="J147:O147"/>
+    <mergeCell ref="B173:G173"/>
+    <mergeCell ref="J173:O173"/>
+    <mergeCell ref="B175:G175"/>
+    <mergeCell ref="J175:O175"/>
+    <mergeCell ref="B231:G231"/>
+    <mergeCell ref="J231:O231"/>
+    <mergeCell ref="B202:G202"/>
+    <mergeCell ref="J202:O202"/>
+    <mergeCell ref="B204:G204"/>
+    <mergeCell ref="J204:O204"/>
+    <mergeCell ref="B233:G233"/>
+    <mergeCell ref="J233:O233"/>
+    <mergeCell ref="B260:G260"/>
+    <mergeCell ref="J260:O260"/>
+    <mergeCell ref="B262:G262"/>
+    <mergeCell ref="J262:O262"/>
+    <mergeCell ref="B289:G289"/>
+    <mergeCell ref="J289:O289"/>
+    <mergeCell ref="B291:G291"/>
+    <mergeCell ref="J291:O291"/>
+    <mergeCell ref="B318:G318"/>
+    <mergeCell ref="J318:O318"/>
+    <mergeCell ref="B320:G320"/>
+    <mergeCell ref="J320:O320"/>
+    <mergeCell ref="B347:G347"/>
+    <mergeCell ref="J347:O347"/>
+    <mergeCell ref="B349:G349"/>
+    <mergeCell ref="J349:O349"/>
+    <mergeCell ref="B434:G434"/>
+    <mergeCell ref="J434:O434"/>
+    <mergeCell ref="B436:G436"/>
+    <mergeCell ref="J436:O436"/>
+    <mergeCell ref="B376:G376"/>
+    <mergeCell ref="J376:O376"/>
+    <mergeCell ref="B378:G378"/>
+    <mergeCell ref="J378:O378"/>
+    <mergeCell ref="B405:G405"/>
+    <mergeCell ref="J405:O405"/>
+    <mergeCell ref="B407:G407"/>
+    <mergeCell ref="J407:O407"/>
+    <mergeCell ref="B520:G520"/>
+    <mergeCell ref="J520:O520"/>
+    <mergeCell ref="B493:G493"/>
+    <mergeCell ref="J493:O493"/>
+    <mergeCell ref="B462:G462"/>
+    <mergeCell ref="J462:O462"/>
+    <mergeCell ref="B464:G464"/>
+    <mergeCell ref="J464:O464"/>
+    <mergeCell ref="B491:G491"/>
+    <mergeCell ref="J491:O491"/>
+    <mergeCell ref="B522:G522"/>
+    <mergeCell ref="J522:O522"/>
+    <mergeCell ref="B549:G549"/>
+    <mergeCell ref="J549:O549"/>
+    <mergeCell ref="B551:G551"/>
+    <mergeCell ref="J551:O551"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>